<commit_message>
Ajusta a tela ao tamanho padrão do Aspen (50 x 35 unidades)
A imagem de 1920 x 1080 (16:9) ficava esticada na tela de 50 x 35
unidades (10:7). Layout refeito em 10:7, imagem em 1400 x 980 e
posições do roteiro e da planilha em unidades do editor.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012cAZJr8EKNEq3XLjv1AThq
</commit_message>
<xml_diff>
--- a/entregaveis/03_aspen/posicoes_objetos.xlsx
+++ b/entregaveis/03_aspen/posicoes_objetos.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="55">
   <si>
-    <t xml:space="preserve">Largura total no editor (passo D4). Deixe 1920 se o editor trabalha em pixels.</t>
+    <t xml:space="preserve">Largura da tela no editor, em unidades (passo C2). O padrão do Aspen é 50.</t>
   </si>
   <si>
     <t xml:space="preserve">Fator de conversão (calculado)</t>
@@ -46,28 +46,28 @@
     <t xml:space="preserve">Atributo</t>
   </si>
   <si>
-    <t xml:space="preserve">X px</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Y px</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Largura px</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Altura px</t>
-  </si>
-  <si>
-    <t xml:space="preserve">X editor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Y editor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Largura editor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Altura editor</t>
+    <t xml:space="preserve">X (tela 50)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Y (tela 50)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Largura (tela 50)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Altura (tela 50)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">X no editor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Y no editor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Largura no editor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Altura no editor</t>
   </si>
   <si>
     <t xml:space="preserve">Fundo</t>
@@ -194,7 +194,7 @@
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
-    <numFmt numFmtId="166" formatCode="General"/>
+    <numFmt numFmtId="166" formatCode="0.00"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -324,7 +324,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -347,6 +347,10 @@
     </xf>
     <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
@@ -624,7 +628,7 @@
         <v>0</v>
       </c>
       <c r="F1" s="2" t="n">
-        <v>1920</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -632,7 +636,7 @@
         <v>1</v>
       </c>
       <c r="F2" s="4" t="n">
-        <f aca="false">F1/1920</f>
+        <f aca="false">F1/50</f>
         <v>1</v>
       </c>
     </row>
@@ -693,33 +697,33 @@
       <c r="D5" s="3"/>
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>
-      <c r="G5" s="3" t="n">
+      <c r="G5" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="H5" s="3" t="n">
+      <c r="H5" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="I5" s="3" t="n">
-        <v>1920</v>
-      </c>
-      <c r="J5" s="3" t="n">
-        <v>1080</v>
-      </c>
-      <c r="K5" s="6" t="n">
-        <f aca="false">ROUND(G5*$F$2,0)</f>
+      <c r="I5" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="K5" s="7" t="n">
+        <f aca="false">ROUND(G5*$F$2,2)</f>
         <v>0</v>
       </c>
-      <c r="L5" s="6" t="n">
-        <f aca="false">ROUND(H5*$F$2,0)</f>
+      <c r="L5" s="7" t="n">
+        <f aca="false">ROUND(H5*$F$2,2)</f>
         <v>0</v>
       </c>
-      <c r="M5" s="6" t="n">
-        <f aca="false">ROUND(I5*$F$2,0)</f>
-        <v>1920</v>
-      </c>
-      <c r="N5" s="6" t="n">
-        <f aca="false">ROUND(J5*$F$2,0)</f>
-        <v>1080</v>
+      <c r="M5" s="7" t="n">
+        <f aca="false">ROUND(I5*$F$2,2)</f>
+        <v>50</v>
+      </c>
+      <c r="N5" s="7" t="n">
+        <f aca="false">ROUND(J5*$F$2,2)</f>
+        <v>35</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -735,33 +739,33 @@
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
-      <c r="G6" s="3" t="n">
-        <v>32</v>
-      </c>
-      <c r="H6" s="3" t="n">
-        <v>16</v>
-      </c>
-      <c r="I6" s="3" t="n">
-        <v>200</v>
-      </c>
-      <c r="J6" s="3" t="n">
-        <v>56</v>
-      </c>
-      <c r="K6" s="6" t="n">
-        <f aca="false">ROUND(G6*$F$2,0)</f>
-        <v>32</v>
-      </c>
-      <c r="L6" s="6" t="n">
-        <f aca="false">ROUND(H6*$F$2,0)</f>
-        <v>16</v>
-      </c>
-      <c r="M6" s="6" t="n">
-        <f aca="false">ROUND(I6*$F$2,0)</f>
-        <v>200</v>
-      </c>
-      <c r="N6" s="6" t="n">
-        <f aca="false">ROUND(J6*$F$2,0)</f>
-        <v>56</v>
+      <c r="G6" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" s="6" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="I6" s="6" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="J6" s="6" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="K6" s="7" t="n">
+        <f aca="false">ROUND(G6*$F$2,2)</f>
+        <v>1</v>
+      </c>
+      <c r="L6" s="7" t="n">
+        <f aca="false">ROUND(H6*$F$2,2)</f>
+        <v>0.48</v>
+      </c>
+      <c r="M6" s="7" t="n">
+        <f aca="false">ROUND(I6*$F$2,2)</f>
+        <v>6.25</v>
+      </c>
+      <c r="N6" s="7" t="n">
+        <f aca="false">ROUND(J6*$F$2,2)</f>
+        <v>1.75</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -783,33 +787,33 @@
       <c r="F7" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="G7" s="3" t="n">
-        <v>1688</v>
-      </c>
-      <c r="H7" s="3" t="n">
-        <v>43</v>
-      </c>
-      <c r="I7" s="3" t="n">
-        <v>200</v>
-      </c>
-      <c r="J7" s="3" t="n">
-        <v>26</v>
-      </c>
-      <c r="K7" s="6" t="n">
-        <f aca="false">ROUND(G7*$F$2,0)</f>
-        <v>1688</v>
-      </c>
-      <c r="L7" s="6" t="n">
-        <f aca="false">ROUND(H7*$F$2,0)</f>
-        <v>43</v>
-      </c>
-      <c r="M7" s="6" t="n">
-        <f aca="false">ROUND(I7*$F$2,0)</f>
-        <v>200</v>
-      </c>
-      <c r="N7" s="6" t="n">
-        <f aca="false">ROUND(J7*$F$2,0)</f>
-        <v>26</v>
+      <c r="G7" s="6" t="n">
+        <v>42.75</v>
+      </c>
+      <c r="H7" s="6" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="I7" s="6" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="J7" s="6" t="n">
+        <v>0.81</v>
+      </c>
+      <c r="K7" s="7" t="n">
+        <f aca="false">ROUND(G7*$F$2,2)</f>
+        <v>42.75</v>
+      </c>
+      <c r="L7" s="7" t="n">
+        <f aca="false">ROUND(H7*$F$2,2)</f>
+        <v>1.34</v>
+      </c>
+      <c r="M7" s="7" t="n">
+        <f aca="false">ROUND(I7*$F$2,2)</f>
+        <v>6.25</v>
+      </c>
+      <c r="N7" s="7" t="n">
+        <f aca="false">ROUND(J7*$F$2,2)</f>
+        <v>0.81</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -831,33 +835,33 @@
       <c r="F8" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="G8" s="3" t="n">
-        <v>57</v>
-      </c>
-      <c r="H8" s="3" t="n">
-        <v>169</v>
-      </c>
-      <c r="I8" s="3" t="n">
-        <v>230</v>
-      </c>
-      <c r="J8" s="3" t="n">
-        <v>84</v>
-      </c>
-      <c r="K8" s="6" t="n">
-        <f aca="false">ROUND(G8*$F$2,0)</f>
-        <v>57</v>
-      </c>
-      <c r="L8" s="6" t="n">
-        <f aca="false">ROUND(H8*$F$2,0)</f>
-        <v>169</v>
-      </c>
-      <c r="M8" s="6" t="n">
-        <f aca="false">ROUND(I8*$F$2,0)</f>
-        <v>230</v>
-      </c>
-      <c r="N8" s="6" t="n">
-        <f aca="false">ROUND(J8*$F$2,0)</f>
-        <v>84</v>
+      <c r="G8" s="6" t="n">
+        <v>1.78</v>
+      </c>
+      <c r="H8" s="6" t="n">
+        <v>5.28</v>
+      </c>
+      <c r="I8" s="6" t="n">
+        <v>6.41</v>
+      </c>
+      <c r="J8" s="6" t="n">
+        <v>2.63</v>
+      </c>
+      <c r="K8" s="7" t="n">
+        <f aca="false">ROUND(G8*$F$2,2)</f>
+        <v>1.78</v>
+      </c>
+      <c r="L8" s="7" t="n">
+        <f aca="false">ROUND(H8*$F$2,2)</f>
+        <v>5.28</v>
+      </c>
+      <c r="M8" s="7" t="n">
+        <f aca="false">ROUND(I8*$F$2,2)</f>
+        <v>6.41</v>
+      </c>
+      <c r="N8" s="7" t="n">
+        <f aca="false">ROUND(J8*$F$2,2)</f>
+        <v>2.63</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -875,33 +879,33 @@
       </c>
       <c r="E9" s="3"/>
       <c r="F9" s="3"/>
-      <c r="G9" s="3" t="n">
-        <v>407</v>
-      </c>
-      <c r="H9" s="3" t="n">
-        <v>176</v>
-      </c>
-      <c r="I9" s="3" t="n">
-        <v>200</v>
-      </c>
-      <c r="J9" s="3" t="n">
-        <v>100</v>
-      </c>
-      <c r="K9" s="6" t="n">
-        <f aca="false">ROUND(G9*$F$2,0)</f>
-        <v>407</v>
-      </c>
-      <c r="L9" s="6" t="n">
-        <f aca="false">ROUND(H9*$F$2,0)</f>
-        <v>176</v>
-      </c>
-      <c r="M9" s="6" t="n">
-        <f aca="false">ROUND(I9*$F$2,0)</f>
-        <v>200</v>
-      </c>
-      <c r="N9" s="6" t="n">
-        <f aca="false">ROUND(J9*$F$2,0)</f>
-        <v>100</v>
+      <c r="G9" s="6" t="n">
+        <v>11.78</v>
+      </c>
+      <c r="H9" s="6" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="I9" s="6" t="n">
+        <v>4.69</v>
+      </c>
+      <c r="J9" s="6" t="n">
+        <v>3.13</v>
+      </c>
+      <c r="K9" s="7" t="n">
+        <f aca="false">ROUND(G9*$F$2,2)</f>
+        <v>11.78</v>
+      </c>
+      <c r="L9" s="7" t="n">
+        <f aca="false">ROUND(H9*$F$2,2)</f>
+        <v>5.5</v>
+      </c>
+      <c r="M9" s="7" t="n">
+        <f aca="false">ROUND(I9*$F$2,2)</f>
+        <v>4.69</v>
+      </c>
+      <c r="N9" s="7" t="n">
+        <f aca="false">ROUND(J9*$F$2,2)</f>
+        <v>3.13</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -923,33 +927,33 @@
       <c r="F10" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="G10" s="3" t="n">
-        <v>159</v>
-      </c>
-      <c r="H10" s="3" t="n">
-        <v>307</v>
-      </c>
-      <c r="I10" s="3" t="n">
-        <v>180</v>
-      </c>
-      <c r="J10" s="3" t="n">
-        <v>22</v>
-      </c>
-      <c r="K10" s="6" t="n">
-        <f aca="false">ROUND(G10*$F$2,0)</f>
-        <v>159</v>
-      </c>
-      <c r="L10" s="6" t="n">
-        <f aca="false">ROUND(H10*$F$2,0)</f>
-        <v>307</v>
-      </c>
-      <c r="M10" s="6" t="n">
-        <f aca="false">ROUND(I10*$F$2,0)</f>
-        <v>180</v>
-      </c>
-      <c r="N10" s="6" t="n">
-        <f aca="false">ROUND(J10*$F$2,0)</f>
-        <v>22</v>
+      <c r="G10" s="6" t="n">
+        <v>4.96</v>
+      </c>
+      <c r="H10" s="6" t="n">
+        <v>9.59</v>
+      </c>
+      <c r="I10" s="6" t="n">
+        <v>5.16</v>
+      </c>
+      <c r="J10" s="6" t="n">
+        <v>0.69</v>
+      </c>
+      <c r="K10" s="7" t="n">
+        <f aca="false">ROUND(G10*$F$2,2)</f>
+        <v>4.96</v>
+      </c>
+      <c r="L10" s="7" t="n">
+        <f aca="false">ROUND(H10*$F$2,2)</f>
+        <v>9.59</v>
+      </c>
+      <c r="M10" s="7" t="n">
+        <f aca="false">ROUND(I10*$F$2,2)</f>
+        <v>5.16</v>
+      </c>
+      <c r="N10" s="7" t="n">
+        <f aca="false">ROUND(J10*$F$2,2)</f>
+        <v>0.69</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -971,33 +975,33 @@
       <c r="F11" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="G11" s="3" t="n">
-        <v>442</v>
-      </c>
-      <c r="H11" s="3" t="n">
-        <v>307</v>
-      </c>
-      <c r="I11" s="3" t="n">
-        <v>90</v>
-      </c>
-      <c r="J11" s="3" t="n">
-        <v>22</v>
-      </c>
-      <c r="K11" s="6" t="n">
-        <f aca="false">ROUND(G11*$F$2,0)</f>
-        <v>442</v>
-      </c>
-      <c r="L11" s="6" t="n">
-        <f aca="false">ROUND(H11*$F$2,0)</f>
-        <v>307</v>
-      </c>
-      <c r="M11" s="6" t="n">
-        <f aca="false">ROUND(I11*$F$2,0)</f>
-        <v>90</v>
-      </c>
-      <c r="N11" s="6" t="n">
-        <f aca="false">ROUND(J11*$F$2,0)</f>
-        <v>22</v>
+      <c r="G11" s="6" t="n">
+        <v>13.08</v>
+      </c>
+      <c r="H11" s="6" t="n">
+        <v>9.59</v>
+      </c>
+      <c r="I11" s="6" t="n">
+        <v>2.81</v>
+      </c>
+      <c r="J11" s="6" t="n">
+        <v>0.69</v>
+      </c>
+      <c r="K11" s="7" t="n">
+        <f aca="false">ROUND(G11*$F$2,2)</f>
+        <v>13.08</v>
+      </c>
+      <c r="L11" s="7" t="n">
+        <f aca="false">ROUND(H11*$F$2,2)</f>
+        <v>9.59</v>
+      </c>
+      <c r="M11" s="7" t="n">
+        <f aca="false">ROUND(I11*$F$2,2)</f>
+        <v>2.81</v>
+      </c>
+      <c r="N11" s="7" t="n">
+        <f aca="false">ROUND(J11*$F$2,2)</f>
+        <v>0.69</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1019,33 +1023,33 @@
       <c r="F12" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="G12" s="3" t="n">
-        <v>677</v>
-      </c>
-      <c r="H12" s="3" t="n">
-        <v>169</v>
-      </c>
-      <c r="I12" s="3" t="n">
-        <v>230</v>
-      </c>
-      <c r="J12" s="3" t="n">
-        <v>84</v>
-      </c>
-      <c r="K12" s="6" t="n">
-        <f aca="false">ROUND(G12*$F$2,0)</f>
-        <v>677</v>
-      </c>
-      <c r="L12" s="6" t="n">
-        <f aca="false">ROUND(H12*$F$2,0)</f>
-        <v>169</v>
-      </c>
-      <c r="M12" s="6" t="n">
-        <f aca="false">ROUND(I12*$F$2,0)</f>
-        <v>230</v>
-      </c>
-      <c r="N12" s="6" t="n">
-        <f aca="false">ROUND(J12*$F$2,0)</f>
-        <v>84</v>
+      <c r="G12" s="6" t="n">
+        <v>18.66</v>
+      </c>
+      <c r="H12" s="6" t="n">
+        <v>5.28</v>
+      </c>
+      <c r="I12" s="6" t="n">
+        <v>6.41</v>
+      </c>
+      <c r="J12" s="6" t="n">
+        <v>2.63</v>
+      </c>
+      <c r="K12" s="7" t="n">
+        <f aca="false">ROUND(G12*$F$2,2)</f>
+        <v>18.66</v>
+      </c>
+      <c r="L12" s="7" t="n">
+        <f aca="false">ROUND(H12*$F$2,2)</f>
+        <v>5.28</v>
+      </c>
+      <c r="M12" s="7" t="n">
+        <f aca="false">ROUND(I12*$F$2,2)</f>
+        <v>6.41</v>
+      </c>
+      <c r="N12" s="7" t="n">
+        <f aca="false">ROUND(J12*$F$2,2)</f>
+        <v>2.63</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1063,33 +1067,33 @@
       </c>
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
-      <c r="G13" s="3" t="n">
-        <v>1027</v>
-      </c>
-      <c r="H13" s="3" t="n">
-        <v>176</v>
-      </c>
-      <c r="I13" s="3" t="n">
-        <v>200</v>
-      </c>
-      <c r="J13" s="3" t="n">
-        <v>100</v>
-      </c>
-      <c r="K13" s="6" t="n">
-        <f aca="false">ROUND(G13*$F$2,0)</f>
-        <v>1027</v>
-      </c>
-      <c r="L13" s="6" t="n">
-        <f aca="false">ROUND(H13*$F$2,0)</f>
-        <v>176</v>
-      </c>
-      <c r="M13" s="6" t="n">
-        <f aca="false">ROUND(I13*$F$2,0)</f>
-        <v>200</v>
-      </c>
-      <c r="N13" s="6" t="n">
-        <f aca="false">ROUND(J13*$F$2,0)</f>
-        <v>100</v>
+      <c r="G13" s="6" t="n">
+        <v>28.66</v>
+      </c>
+      <c r="H13" s="6" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="I13" s="6" t="n">
+        <v>4.69</v>
+      </c>
+      <c r="J13" s="6" t="n">
+        <v>3.13</v>
+      </c>
+      <c r="K13" s="7" t="n">
+        <f aca="false">ROUND(G13*$F$2,2)</f>
+        <v>28.66</v>
+      </c>
+      <c r="L13" s="7" t="n">
+        <f aca="false">ROUND(H13*$F$2,2)</f>
+        <v>5.5</v>
+      </c>
+      <c r="M13" s="7" t="n">
+        <f aca="false">ROUND(I13*$F$2,2)</f>
+        <v>4.69</v>
+      </c>
+      <c r="N13" s="7" t="n">
+        <f aca="false">ROUND(J13*$F$2,2)</f>
+        <v>3.13</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1111,33 +1115,33 @@
       <c r="F14" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="G14" s="3" t="n">
-        <v>779</v>
-      </c>
-      <c r="H14" s="3" t="n">
-        <v>307</v>
-      </c>
-      <c r="I14" s="3" t="n">
-        <v>180</v>
-      </c>
-      <c r="J14" s="3" t="n">
-        <v>22</v>
-      </c>
-      <c r="K14" s="6" t="n">
-        <f aca="false">ROUND(G14*$F$2,0)</f>
-        <v>779</v>
-      </c>
-      <c r="L14" s="6" t="n">
-        <f aca="false">ROUND(H14*$F$2,0)</f>
-        <v>307</v>
-      </c>
-      <c r="M14" s="6" t="n">
-        <f aca="false">ROUND(I14*$F$2,0)</f>
-        <v>180</v>
-      </c>
-      <c r="N14" s="6" t="n">
-        <f aca="false">ROUND(J14*$F$2,0)</f>
-        <v>22</v>
+      <c r="G14" s="6" t="n">
+        <v>21.84</v>
+      </c>
+      <c r="H14" s="6" t="n">
+        <v>9.59</v>
+      </c>
+      <c r="I14" s="6" t="n">
+        <v>5.16</v>
+      </c>
+      <c r="J14" s="6" t="n">
+        <v>0.69</v>
+      </c>
+      <c r="K14" s="7" t="n">
+        <f aca="false">ROUND(G14*$F$2,2)</f>
+        <v>21.84</v>
+      </c>
+      <c r="L14" s="7" t="n">
+        <f aca="false">ROUND(H14*$F$2,2)</f>
+        <v>9.59</v>
+      </c>
+      <c r="M14" s="7" t="n">
+        <f aca="false">ROUND(I14*$F$2,2)</f>
+        <v>5.16</v>
+      </c>
+      <c r="N14" s="7" t="n">
+        <f aca="false">ROUND(J14*$F$2,2)</f>
+        <v>0.69</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1159,33 +1163,33 @@
       <c r="F15" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="G15" s="3" t="n">
-        <v>1062</v>
-      </c>
-      <c r="H15" s="3" t="n">
-        <v>307</v>
-      </c>
-      <c r="I15" s="3" t="n">
-        <v>90</v>
-      </c>
-      <c r="J15" s="3" t="n">
-        <v>22</v>
-      </c>
-      <c r="K15" s="6" t="n">
-        <f aca="false">ROUND(G15*$F$2,0)</f>
-        <v>1062</v>
-      </c>
-      <c r="L15" s="6" t="n">
-        <f aca="false">ROUND(H15*$F$2,0)</f>
-        <v>307</v>
-      </c>
-      <c r="M15" s="6" t="n">
-        <f aca="false">ROUND(I15*$F$2,0)</f>
-        <v>90</v>
-      </c>
-      <c r="N15" s="6" t="n">
-        <f aca="false">ROUND(J15*$F$2,0)</f>
-        <v>22</v>
+      <c r="G15" s="6" t="n">
+        <v>29.96</v>
+      </c>
+      <c r="H15" s="6" t="n">
+        <v>9.59</v>
+      </c>
+      <c r="I15" s="6" t="n">
+        <v>2.81</v>
+      </c>
+      <c r="J15" s="6" t="n">
+        <v>0.69</v>
+      </c>
+      <c r="K15" s="7" t="n">
+        <f aca="false">ROUND(G15*$F$2,2)</f>
+        <v>29.96</v>
+      </c>
+      <c r="L15" s="7" t="n">
+        <f aca="false">ROUND(H15*$F$2,2)</f>
+        <v>9.59</v>
+      </c>
+      <c r="M15" s="7" t="n">
+        <f aca="false">ROUND(I15*$F$2,2)</f>
+        <v>2.81</v>
+      </c>
+      <c r="N15" s="7" t="n">
+        <f aca="false">ROUND(J15*$F$2,2)</f>
+        <v>0.69</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1207,33 +1211,33 @@
       <c r="F16" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="G16" s="3" t="n">
-        <v>1297</v>
-      </c>
-      <c r="H16" s="3" t="n">
-        <v>188</v>
-      </c>
-      <c r="I16" s="3" t="n">
-        <v>170</v>
-      </c>
-      <c r="J16" s="3" t="n">
-        <v>84</v>
-      </c>
-      <c r="K16" s="6" t="n">
-        <f aca="false">ROUND(G16*$F$2,0)</f>
-        <v>1297</v>
-      </c>
-      <c r="L16" s="6" t="n">
-        <f aca="false">ROUND(H16*$F$2,0)</f>
-        <v>188</v>
-      </c>
-      <c r="M16" s="6" t="n">
-        <f aca="false">ROUND(I16*$F$2,0)</f>
-        <v>170</v>
-      </c>
-      <c r="N16" s="6" t="n">
-        <f aca="false">ROUND(J16*$F$2,0)</f>
-        <v>84</v>
+      <c r="G16" s="6" t="n">
+        <v>35.53</v>
+      </c>
+      <c r="H16" s="6" t="n">
+        <v>5.88</v>
+      </c>
+      <c r="I16" s="6" t="n">
+        <v>5.31</v>
+      </c>
+      <c r="J16" s="6" t="n">
+        <v>2.63</v>
+      </c>
+      <c r="K16" s="7" t="n">
+        <f aca="false">ROUND(G16*$F$2,2)</f>
+        <v>35.53</v>
+      </c>
+      <c r="L16" s="7" t="n">
+        <f aca="false">ROUND(H16*$F$2,2)</f>
+        <v>5.88</v>
+      </c>
+      <c r="M16" s="7" t="n">
+        <f aca="false">ROUND(I16*$F$2,2)</f>
+        <v>5.31</v>
+      </c>
+      <c r="N16" s="7" t="n">
+        <f aca="false">ROUND(J16*$F$2,2)</f>
+        <v>2.63</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1255,33 +1259,33 @@
       <c r="F17" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="G17" s="3" t="n">
-        <v>1398</v>
-      </c>
-      <c r="H17" s="3" t="n">
-        <v>303</v>
-      </c>
-      <c r="I17" s="3" t="n">
-        <v>150</v>
-      </c>
-      <c r="J17" s="3" t="n">
-        <v>22</v>
-      </c>
-      <c r="K17" s="6" t="n">
-        <f aca="false">ROUND(G17*$F$2,0)</f>
-        <v>1398</v>
-      </c>
-      <c r="L17" s="6" t="n">
-        <f aca="false">ROUND(H17*$F$2,0)</f>
-        <v>303</v>
-      </c>
-      <c r="M17" s="6" t="n">
-        <f aca="false">ROUND(I17*$F$2,0)</f>
-        <v>150</v>
-      </c>
-      <c r="N17" s="6" t="n">
-        <f aca="false">ROUND(J17*$F$2,0)</f>
-        <v>22</v>
+      <c r="G17" s="6" t="n">
+        <v>43.53</v>
+      </c>
+      <c r="H17" s="6" t="n">
+        <v>8.75</v>
+      </c>
+      <c r="I17" s="6" t="n">
+        <v>4.69</v>
+      </c>
+      <c r="J17" s="6" t="n">
+        <v>0.69</v>
+      </c>
+      <c r="K17" s="7" t="n">
+        <f aca="false">ROUND(G17*$F$2,2)</f>
+        <v>43.53</v>
+      </c>
+      <c r="L17" s="7" t="n">
+        <f aca="false">ROUND(H17*$F$2,2)</f>
+        <v>8.75</v>
+      </c>
+      <c r="M17" s="7" t="n">
+        <f aca="false">ROUND(I17*$F$2,2)</f>
+        <v>4.69</v>
+      </c>
+      <c r="N17" s="7" t="n">
+        <f aca="false">ROUND(J17*$F$2,2)</f>
+        <v>0.69</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1303,33 +1307,33 @@
       <c r="F18" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="G18" s="3" t="n">
-        <v>1753</v>
-      </c>
-      <c r="H18" s="3" t="n">
-        <v>200</v>
-      </c>
-      <c r="I18" s="3" t="n">
-        <v>110</v>
-      </c>
-      <c r="J18" s="3" t="n">
-        <v>26</v>
-      </c>
-      <c r="K18" s="6" t="n">
-        <f aca="false">ROUND(G18*$F$2,0)</f>
-        <v>1753</v>
-      </c>
-      <c r="L18" s="6" t="n">
-        <f aca="false">ROUND(H18*$F$2,0)</f>
-        <v>200</v>
-      </c>
-      <c r="M18" s="6" t="n">
-        <f aca="false">ROUND(I18*$F$2,0)</f>
-        <v>110</v>
-      </c>
-      <c r="N18" s="6" t="n">
-        <f aca="false">ROUND(J18*$F$2,0)</f>
-        <v>26</v>
+      <c r="G18" s="6" t="n">
+        <v>44.78</v>
+      </c>
+      <c r="H18" s="6" t="n">
+        <v>11.31</v>
+      </c>
+      <c r="I18" s="6" t="n">
+        <v>3.44</v>
+      </c>
+      <c r="J18" s="6" t="n">
+        <v>0.81</v>
+      </c>
+      <c r="K18" s="7" t="n">
+        <f aca="false">ROUND(G18*$F$2,2)</f>
+        <v>44.78</v>
+      </c>
+      <c r="L18" s="7" t="n">
+        <f aca="false">ROUND(H18*$F$2,2)</f>
+        <v>11.31</v>
+      </c>
+      <c r="M18" s="7" t="n">
+        <f aca="false">ROUND(I18*$F$2,2)</f>
+        <v>3.44</v>
+      </c>
+      <c r="N18" s="7" t="n">
+        <f aca="false">ROUND(J18*$F$2,2)</f>
+        <v>0.81</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1351,33 +1355,33 @@
       <c r="F19" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="G19" s="3" t="n">
-        <v>1753</v>
-      </c>
-      <c r="H19" s="3" t="n">
-        <v>240</v>
-      </c>
-      <c r="I19" s="3" t="n">
-        <v>110</v>
-      </c>
-      <c r="J19" s="3" t="n">
-        <v>26</v>
-      </c>
-      <c r="K19" s="6" t="n">
-        <f aca="false">ROUND(G19*$F$2,0)</f>
-        <v>1753</v>
-      </c>
-      <c r="L19" s="6" t="n">
-        <f aca="false">ROUND(H19*$F$2,0)</f>
-        <v>240</v>
-      </c>
-      <c r="M19" s="6" t="n">
-        <f aca="false">ROUND(I19*$F$2,0)</f>
-        <v>110</v>
-      </c>
-      <c r="N19" s="6" t="n">
-        <f aca="false">ROUND(J19*$F$2,0)</f>
-        <v>26</v>
+      <c r="G19" s="6" t="n">
+        <v>44.78</v>
+      </c>
+      <c r="H19" s="6" t="n">
+        <v>12.56</v>
+      </c>
+      <c r="I19" s="6" t="n">
+        <v>3.44</v>
+      </c>
+      <c r="J19" s="6" t="n">
+        <v>0.81</v>
+      </c>
+      <c r="K19" s="7" t="n">
+        <f aca="false">ROUND(G19*$F$2,2)</f>
+        <v>44.78</v>
+      </c>
+      <c r="L19" s="7" t="n">
+        <f aca="false">ROUND(H19*$F$2,2)</f>
+        <v>12.56</v>
+      </c>
+      <c r="M19" s="7" t="n">
+        <f aca="false">ROUND(I19*$F$2,2)</f>
+        <v>3.44</v>
+      </c>
+      <c r="N19" s="7" t="n">
+        <f aca="false">ROUND(J19*$F$2,2)</f>
+        <v>0.81</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1395,33 +1399,33 @@
       </c>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
-      <c r="G20" s="3" t="n">
-        <v>57</v>
-      </c>
-      <c r="H20" s="3" t="n">
-        <v>468</v>
-      </c>
-      <c r="I20" s="3" t="n">
-        <v>1290</v>
-      </c>
-      <c r="J20" s="3" t="n">
-        <v>560</v>
-      </c>
-      <c r="K20" s="6" t="n">
-        <f aca="false">ROUND(G20*$F$2,0)</f>
-        <v>57</v>
-      </c>
-      <c r="L20" s="6" t="n">
-        <f aca="false">ROUND(H20*$F$2,0)</f>
-        <v>468</v>
-      </c>
-      <c r="M20" s="6" t="n">
-        <f aca="false">ROUND(I20*$F$2,0)</f>
-        <v>1290</v>
-      </c>
-      <c r="N20" s="6" t="n">
-        <f aca="false">ROUND(J20*$F$2,0)</f>
-        <v>560</v>
+      <c r="G20" s="6" t="n">
+        <v>1.78</v>
+      </c>
+      <c r="H20" s="6" t="n">
+        <v>14.63</v>
+      </c>
+      <c r="I20" s="6" t="n">
+        <v>31.63</v>
+      </c>
+      <c r="J20" s="6" t="n">
+        <v>18.63</v>
+      </c>
+      <c r="K20" s="7" t="n">
+        <f aca="false">ROUND(G20*$F$2,2)</f>
+        <v>1.78</v>
+      </c>
+      <c r="L20" s="7" t="n">
+        <f aca="false">ROUND(H20*$F$2,2)</f>
+        <v>14.63</v>
+      </c>
+      <c r="M20" s="7" t="n">
+        <f aca="false">ROUND(I20*$F$2,2)</f>
+        <v>31.63</v>
+      </c>
+      <c r="N20" s="7" t="n">
+        <f aca="false">ROUND(J20*$F$2,2)</f>
+        <v>18.63</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1443,33 +1447,33 @@
       <c r="F21" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="G21" s="3" t="n">
-        <v>1710</v>
-      </c>
-      <c r="H21" s="3" t="n">
-        <v>512</v>
-      </c>
-      <c r="I21" s="3" t="n">
-        <v>130</v>
-      </c>
-      <c r="J21" s="3" t="n">
-        <v>32</v>
-      </c>
-      <c r="K21" s="6" t="n">
-        <f aca="false">ROUND(G21*$F$2,0)</f>
-        <v>1710</v>
-      </c>
-      <c r="L21" s="6" t="n">
-        <f aca="false">ROUND(H21*$F$2,0)</f>
-        <v>512</v>
-      </c>
-      <c r="M21" s="6" t="n">
-        <f aca="false">ROUND(I21*$F$2,0)</f>
-        <v>130</v>
-      </c>
-      <c r="N21" s="6" t="n">
-        <f aca="false">ROUND(J21*$F$2,0)</f>
-        <v>32</v>
+      <c r="G21" s="6" t="n">
+        <v>44.31</v>
+      </c>
+      <c r="H21" s="6" t="n">
+        <v>19.94</v>
+      </c>
+      <c r="I21" s="6" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="J21" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="K21" s="7" t="n">
+        <f aca="false">ROUND(G21*$F$2,2)</f>
+        <v>44.31</v>
+      </c>
+      <c r="L21" s="7" t="n">
+        <f aca="false">ROUND(H21*$F$2,2)</f>
+        <v>19.94</v>
+      </c>
+      <c r="M21" s="7" t="n">
+        <f aca="false">ROUND(I21*$F$2,2)</f>
+        <v>3.25</v>
+      </c>
+      <c r="N21" s="7" t="n">
+        <f aca="false">ROUND(J21*$F$2,2)</f>
+        <v>1</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1491,33 +1495,33 @@
       <c r="F22" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="G22" s="3" t="n">
-        <v>1710</v>
-      </c>
-      <c r="H22" s="3" t="n">
-        <v>686</v>
-      </c>
-      <c r="I22" s="3" t="n">
-        <v>130</v>
-      </c>
-      <c r="J22" s="3" t="n">
-        <v>32</v>
-      </c>
-      <c r="K22" s="6" t="n">
-        <f aca="false">ROUND(G22*$F$2,0)</f>
-        <v>1710</v>
-      </c>
-      <c r="L22" s="6" t="n">
-        <f aca="false">ROUND(H22*$F$2,0)</f>
-        <v>686</v>
-      </c>
-      <c r="M22" s="6" t="n">
-        <f aca="false">ROUND(I22*$F$2,0)</f>
-        <v>130</v>
-      </c>
-      <c r="N22" s="6" t="n">
-        <f aca="false">ROUND(J22*$F$2,0)</f>
-        <v>32</v>
+      <c r="G22" s="6" t="n">
+        <v>44.31</v>
+      </c>
+      <c r="H22" s="6" t="n">
+        <v>24.56</v>
+      </c>
+      <c r="I22" s="6" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="J22" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="K22" s="7" t="n">
+        <f aca="false">ROUND(G22*$F$2,2)</f>
+        <v>44.31</v>
+      </c>
+      <c r="L22" s="7" t="n">
+        <f aca="false">ROUND(H22*$F$2,2)</f>
+        <v>24.56</v>
+      </c>
+      <c r="M22" s="7" t="n">
+        <f aca="false">ROUND(I22*$F$2,2)</f>
+        <v>3.25</v>
+      </c>
+      <c r="N22" s="7" t="n">
+        <f aca="false">ROUND(J22*$F$2,2)</f>
+        <v>1</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1539,33 +1543,33 @@
       <c r="F23" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="G23" s="3" t="n">
-        <v>1710</v>
-      </c>
-      <c r="H23" s="3" t="n">
-        <v>860</v>
-      </c>
-      <c r="I23" s="3" t="n">
-        <v>130</v>
-      </c>
-      <c r="J23" s="3" t="n">
-        <v>32</v>
-      </c>
-      <c r="K23" s="6" t="n">
-        <f aca="false">ROUND(G23*$F$2,0)</f>
-        <v>1710</v>
-      </c>
-      <c r="L23" s="6" t="n">
-        <f aca="false">ROUND(H23*$F$2,0)</f>
-        <v>860</v>
-      </c>
-      <c r="M23" s="6" t="n">
-        <f aca="false">ROUND(I23*$F$2,0)</f>
-        <v>130</v>
-      </c>
-      <c r="N23" s="6" t="n">
-        <f aca="false">ROUND(J23*$F$2,0)</f>
-        <v>32</v>
+      <c r="G23" s="6" t="n">
+        <v>44.31</v>
+      </c>
+      <c r="H23" s="6" t="n">
+        <v>29.19</v>
+      </c>
+      <c r="I23" s="6" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="J23" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="K23" s="7" t="n">
+        <f aca="false">ROUND(G23*$F$2,2)</f>
+        <v>44.31</v>
+      </c>
+      <c r="L23" s="7" t="n">
+        <f aca="false">ROUND(H23*$F$2,2)</f>
+        <v>29.19</v>
+      </c>
+      <c r="M23" s="7" t="n">
+        <f aca="false">ROUND(I23*$F$2,2)</f>
+        <v>3.25</v>
+      </c>
+      <c r="N23" s="7" t="n">
+        <f aca="false">ROUND(J23*$F$2,2)</f>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Gera a tela direto em .atgraphic com objetos nativos do Aspen
A imagem de fundo perdia nitidez ao maximizar. A tela passa a ser um
arquivo .atgraphic gerado no formato da tela PQ US04 (painéis, textos,
campos de dados e tendências nativos), com arquivo mínimo de
diagnóstico, conferência por releitura e roteiro reescrito.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012cAZJr8EKNEq3XLjv1AThq
</commit_message>
<xml_diff>
--- a/entregaveis/03_aspen/posicoes_objetos.xlsx
+++ b/entregaveis/03_aspen/posicoes_objetos.xlsx
@@ -20,9 +20,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="55">
-  <si>
-    <t xml:space="preserve">Largura da tela no editor, em unidades (passo C2). O padrão do Aspen é 50.</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="56">
+  <si>
+    <t xml:space="preserve">Largura da tela no editor, em unidades. O padrão do Aspen é 50; só altere se a tela tiver outro tamanho.</t>
   </si>
   <si>
     <t xml:space="preserve">Fator de conversão (calculado)</t>
@@ -70,18 +70,21 @@
     <t xml:space="preserve">Altura no editor</t>
   </si>
   <si>
-    <t xml:space="preserve">Fundo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Imagem de fundo ou mapa</t>
+    <t xml:space="preserve">Tela</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tela inteira (referência)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Logotipo oficial</t>
   </si>
   <si>
     <t xml:space="preserve">Imagem</t>
   </si>
   <si>
-    <t xml:space="preserve">Logotipo oficial</t>
-  </si>
-  <si>
     <t xml:space="preserve">Última atualização (cabeçalho)</t>
   </si>
   <si>
@@ -94,7 +97,7 @@
     <t xml:space="preserve">IP_ANALOGMAP</t>
   </si>
   <si>
-    <t xml:space="preserve">ATRIBUTO DE HORA (anotado em B3)</t>
+    <t xml:space="preserve">`VAL` no arquivo: trocar pelo atributo de data e hora (Parte B)</t>
   </si>
   <si>
     <t xml:space="preserve">Carga média: valor</t>
@@ -115,7 +118,7 @@
     <t xml:space="preserve">Carga média: qualidade</t>
   </si>
   <si>
-    <t xml:space="preserve">ATRIBUTO DE QUALIDADE (anotado em B3)</t>
+    <t xml:space="preserve">`VAL` no arquivo: trocar pelo atributo de qualidade (Parte B)</t>
   </si>
   <si>
     <t xml:space="preserve">Desvio padrão: valor</t>
@@ -172,7 +175,7 @@
     <t xml:space="preserve">307-QI-003</t>
   </si>
   <si>
-    <t xml:space="preserve">mapa de discreto anotado em B4 (provavelmente IP_DISCRETEMAP)</t>
+    <t xml:space="preserve">IP_DISCRETEMAP no arquivo: **conferir** (Parte B)</t>
   </si>
   <si>
     <t xml:space="preserve">Faixa menor que 150 (Alerta)</t>
@@ -734,7 +737,7 @@
         <v>19</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
@@ -773,25 +776,25 @@
         <v>2</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G7" s="6" t="n">
         <v>42.75</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>1.34</v>
+        <v>1.31</v>
       </c>
       <c r="I7" s="6" t="n">
         <v>6.25</v>
@@ -805,7 +808,7 @@
       </c>
       <c r="L7" s="7" t="n">
         <f aca="false">ROUND(H7*$F$2,2)</f>
-        <v>1.34</v>
+        <v>1.31</v>
       </c>
       <c r="M7" s="7" t="n">
         <f aca="false">ROUND(I7*$F$2,2)</f>
@@ -821,25 +824,25 @@
         <v>3</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G8" s="6" t="n">
         <v>1.78</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>5.28</v>
+        <v>5.25</v>
       </c>
       <c r="I8" s="6" t="n">
         <v>6.41</v>
@@ -853,7 +856,7 @@
       </c>
       <c r="L8" s="7" t="n">
         <f aca="false">ROUND(H8*$F$2,2)</f>
-        <v>5.28</v>
+        <v>5.25</v>
       </c>
       <c r="M8" s="7" t="n">
         <f aca="false">ROUND(I8*$F$2,2)</f>
@@ -869,13 +872,13 @@
         <v>4</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E9" s="3"/>
       <c r="F9" s="3"/>
@@ -883,7 +886,7 @@
         <v>11.78</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>5.5</v>
+        <v>5.44</v>
       </c>
       <c r="I9" s="6" t="n">
         <v>4.69</v>
@@ -897,7 +900,7 @@
       </c>
       <c r="L9" s="7" t="n">
         <f aca="false">ROUND(H9*$F$2,2)</f>
-        <v>5.5</v>
+        <v>5.44</v>
       </c>
       <c r="M9" s="7" t="n">
         <f aca="false">ROUND(I9*$F$2,2)</f>
@@ -913,25 +916,25 @@
         <v>5</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>4.96</v>
+        <v>4.8</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>9.59</v>
+        <v>9.53</v>
       </c>
       <c r="I10" s="6" t="n">
         <v>5.16</v>
@@ -941,11 +944,11 @@
       </c>
       <c r="K10" s="7" t="n">
         <f aca="false">ROUND(G10*$F$2,2)</f>
-        <v>4.96</v>
+        <v>4.8</v>
       </c>
       <c r="L10" s="7" t="n">
         <f aca="false">ROUND(H10*$F$2,2)</f>
-        <v>9.59</v>
+        <v>9.53</v>
       </c>
       <c r="M10" s="7" t="n">
         <f aca="false">ROUND(I10*$F$2,2)</f>
@@ -961,25 +964,25 @@
         <v>6</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>13.08</v>
+        <v>12.83</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>9.59</v>
+        <v>9.53</v>
       </c>
       <c r="I11" s="6" t="n">
         <v>2.81</v>
@@ -989,11 +992,11 @@
       </c>
       <c r="K11" s="7" t="n">
         <f aca="false">ROUND(G11*$F$2,2)</f>
-        <v>13.08</v>
+        <v>12.83</v>
       </c>
       <c r="L11" s="7" t="n">
         <f aca="false">ROUND(H11*$F$2,2)</f>
-        <v>9.59</v>
+        <v>9.53</v>
       </c>
       <c r="M11" s="7" t="n">
         <f aca="false">ROUND(I11*$F$2,2)</f>
@@ -1009,25 +1012,25 @@
         <v>7</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G12" s="6" t="n">
         <v>18.66</v>
       </c>
       <c r="H12" s="6" t="n">
-        <v>5.28</v>
+        <v>5.25</v>
       </c>
       <c r="I12" s="6" t="n">
         <v>6.41</v>
@@ -1041,7 +1044,7 @@
       </c>
       <c r="L12" s="7" t="n">
         <f aca="false">ROUND(H12*$F$2,2)</f>
-        <v>5.28</v>
+        <v>5.25</v>
       </c>
       <c r="M12" s="7" t="n">
         <f aca="false">ROUND(I12*$F$2,2)</f>
@@ -1057,13 +1060,13 @@
         <v>8</v>
       </c>
       <c r="B13" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D13" s="3" t="s">
         <v>34</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>33</v>
       </c>
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
@@ -1071,7 +1074,7 @@
         <v>28.66</v>
       </c>
       <c r="H13" s="6" t="n">
-        <v>5.5</v>
+        <v>5.44</v>
       </c>
       <c r="I13" s="6" t="n">
         <v>4.69</v>
@@ -1085,7 +1088,7 @@
       </c>
       <c r="L13" s="7" t="n">
         <f aca="false">ROUND(H13*$F$2,2)</f>
-        <v>5.5</v>
+        <v>5.44</v>
       </c>
       <c r="M13" s="7" t="n">
         <f aca="false">ROUND(I13*$F$2,2)</f>
@@ -1101,25 +1104,25 @@
         <v>9</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>21.84</v>
+        <v>21.68</v>
       </c>
       <c r="H14" s="6" t="n">
-        <v>9.59</v>
+        <v>9.53</v>
       </c>
       <c r="I14" s="6" t="n">
         <v>5.16</v>
@@ -1129,11 +1132,11 @@
       </c>
       <c r="K14" s="7" t="n">
         <f aca="false">ROUND(G14*$F$2,2)</f>
-        <v>21.84</v>
+        <v>21.68</v>
       </c>
       <c r="L14" s="7" t="n">
         <f aca="false">ROUND(H14*$F$2,2)</f>
-        <v>9.59</v>
+        <v>9.53</v>
       </c>
       <c r="M14" s="7" t="n">
         <f aca="false">ROUND(I14*$F$2,2)</f>
@@ -1149,25 +1152,25 @@
         <v>10</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G15" s="6" t="n">
-        <v>29.96</v>
+        <v>29.7</v>
       </c>
       <c r="H15" s="6" t="n">
-        <v>9.59</v>
+        <v>9.53</v>
       </c>
       <c r="I15" s="6" t="n">
         <v>2.81</v>
@@ -1177,11 +1180,11 @@
       </c>
       <c r="K15" s="7" t="n">
         <f aca="false">ROUND(G15*$F$2,2)</f>
-        <v>29.96</v>
+        <v>29.7</v>
       </c>
       <c r="L15" s="7" t="n">
         <f aca="false">ROUND(H15*$F$2,2)</f>
-        <v>9.59</v>
+        <v>9.53</v>
       </c>
       <c r="M15" s="7" t="n">
         <f aca="false">ROUND(I15*$F$2,2)</f>
@@ -1197,25 +1200,25 @@
         <v>11</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G16" s="6" t="n">
         <v>35.53</v>
       </c>
       <c r="H16" s="6" t="n">
-        <v>5.88</v>
+        <v>5.81</v>
       </c>
       <c r="I16" s="6" t="n">
         <v>5.31</v>
@@ -1229,7 +1232,7 @@
       </c>
       <c r="L16" s="7" t="n">
         <f aca="false">ROUND(H16*$F$2,2)</f>
-        <v>5.88</v>
+        <v>5.81</v>
       </c>
       <c r="M16" s="7" t="n">
         <f aca="false">ROUND(I16*$F$2,2)</f>
@@ -1245,25 +1248,25 @@
         <v>12</v>
       </c>
       <c r="B17" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="E17" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="C17" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>39</v>
-      </c>
       <c r="F17" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G17" s="6" t="n">
         <v>43.53</v>
       </c>
       <c r="H17" s="6" t="n">
-        <v>8.75</v>
+        <v>8.69</v>
       </c>
       <c r="I17" s="6" t="n">
         <v>4.69</v>
@@ -1277,7 +1280,7 @@
       </c>
       <c r="L17" s="7" t="n">
         <f aca="false">ROUND(H17*$F$2,2)</f>
-        <v>8.75</v>
+        <v>8.69</v>
       </c>
       <c r="M17" s="7" t="n">
         <f aca="false">ROUND(I17*$F$2,2)</f>
@@ -1293,25 +1296,25 @@
         <v>13</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G18" s="6" t="n">
         <v>44.78</v>
       </c>
       <c r="H18" s="6" t="n">
-        <v>11.31</v>
+        <v>11.22</v>
       </c>
       <c r="I18" s="6" t="n">
         <v>3.44</v>
@@ -1325,7 +1328,7 @@
       </c>
       <c r="L18" s="7" t="n">
         <f aca="false">ROUND(H18*$F$2,2)</f>
-        <v>11.31</v>
+        <v>11.22</v>
       </c>
       <c r="M18" s="7" t="n">
         <f aca="false">ROUND(I18*$F$2,2)</f>
@@ -1341,25 +1344,25 @@
         <v>14</v>
       </c>
       <c r="B19" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="E19" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C19" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="D19" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>43</v>
-      </c>
       <c r="F19" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G19" s="6" t="n">
         <v>44.78</v>
       </c>
       <c r="H19" s="6" t="n">
-        <v>12.56</v>
+        <v>12.47</v>
       </c>
       <c r="I19" s="6" t="n">
         <v>3.44</v>
@@ -1373,7 +1376,7 @@
       </c>
       <c r="L19" s="7" t="n">
         <f aca="false">ROUND(H19*$F$2,2)</f>
-        <v>12.56</v>
+        <v>12.47</v>
       </c>
       <c r="M19" s="7" t="n">
         <f aca="false">ROUND(I19*$F$2,2)</f>
@@ -1389,31 +1392,31 @@
         <v>15</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
       <c r="G20" s="6" t="n">
-        <v>1.78</v>
+        <v>3.03</v>
       </c>
       <c r="H20" s="6" t="n">
         <v>14.63</v>
       </c>
       <c r="I20" s="6" t="n">
-        <v>31.63</v>
+        <v>29.63</v>
       </c>
       <c r="J20" s="6" t="n">
-        <v>18.63</v>
+        <v>18</v>
       </c>
       <c r="K20" s="7" t="n">
         <f aca="false">ROUND(G20*$F$2,2)</f>
-        <v>1.78</v>
+        <v>3.03</v>
       </c>
       <c r="L20" s="7" t="n">
         <f aca="false">ROUND(H20*$F$2,2)</f>
@@ -1421,11 +1424,11 @@
       </c>
       <c r="M20" s="7" t="n">
         <f aca="false">ROUND(I20*$F$2,2)</f>
-        <v>31.63</v>
+        <v>29.63</v>
       </c>
       <c r="N20" s="7" t="n">
         <f aca="false">ROUND(J20*$F$2,2)</f>
-        <v>18.63</v>
+        <v>18</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1433,25 +1436,25 @@
         <v>16</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G21" s="6" t="n">
         <v>44.31</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>19.94</v>
+        <v>19.91</v>
       </c>
       <c r="I21" s="6" t="n">
         <v>3.25</v>
@@ -1465,7 +1468,7 @@
       </c>
       <c r="L21" s="7" t="n">
         <f aca="false">ROUND(H21*$F$2,2)</f>
-        <v>19.94</v>
+        <v>19.91</v>
       </c>
       <c r="M21" s="7" t="n">
         <f aca="false">ROUND(I21*$F$2,2)</f>
@@ -1481,25 +1484,25 @@
         <v>17</v>
       </c>
       <c r="B22" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="E22" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="C22" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="D22" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="E22" s="3" t="s">
-        <v>50</v>
-      </c>
       <c r="F22" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G22" s="6" t="n">
         <v>44.31</v>
       </c>
       <c r="H22" s="6" t="n">
-        <v>24.56</v>
+        <v>24.53</v>
       </c>
       <c r="I22" s="6" t="n">
         <v>3.25</v>
@@ -1513,7 +1516,7 @@
       </c>
       <c r="L22" s="7" t="n">
         <f aca="false">ROUND(H22*$F$2,2)</f>
-        <v>24.56</v>
+        <v>24.53</v>
       </c>
       <c r="M22" s="7" t="n">
         <f aca="false">ROUND(I22*$F$2,2)</f>
@@ -1529,25 +1532,25 @@
         <v>18</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G23" s="6" t="n">
         <v>44.31</v>
       </c>
       <c r="H23" s="6" t="n">
-        <v>29.19</v>
+        <v>29.16</v>
       </c>
       <c r="I23" s="6" t="n">
         <v>3.25</v>
@@ -1561,7 +1564,7 @@
       </c>
       <c r="L23" s="7" t="n">
         <f aca="false">ROUND(H23*$F$2,2)</f>
-        <v>29.19</v>
+        <v>29.16</v>
       </c>
       <c r="M23" s="7" t="n">
         <f aca="false">ROUND(I23*$F$2,2)</f>

</xml_diff>

<commit_message>
Gera a tela v6 em .atgraphic com logotipo, lâmpadas e composto de 2 h
Logotipo oficial em polígonos, lâmpadas animadas no padrão da tela PQ
US04, tendência com ensaios, composto da prensa e composto do
laboratório, campos ligados às tags calculadas do composto e escrita
OLE com várias tabelas de alocação.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012cAZJr8EKNEq3XLjv1AThq
</commit_message>
<xml_diff>
--- a/entregaveis/03_aspen/posicoes_objetos.xlsx
+++ b/entregaveis/03_aspen/posicoes_objetos.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="65">
   <si>
     <t xml:space="preserve">Largura da tela no editor, em unidades. O padrão do Aspen é 50; só altere se a tela tiver outro tamanho.</t>
   </si>
@@ -79,12 +79,6 @@
     <t xml:space="preserve">-</t>
   </si>
   <si>
-    <t xml:space="preserve">Logotipo oficial</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Imagem</t>
-  </si>
-  <si>
     <t xml:space="preserve">Última atualização (cabeçalho)</t>
   </si>
   <si>
@@ -100,22 +94,22 @@
     <t xml:space="preserve">`VAL` no arquivo: trocar pelo atributo de data e hora (Parte B)</t>
   </si>
   <si>
-    <t xml:space="preserve">Carga média: valor</t>
+    <t xml:space="preserve">Média prensa automática: valor</t>
   </si>
   <si>
     <t xml:space="preserve">VAL</t>
   </si>
   <si>
-    <t xml:space="preserve">Carga média: minitendência</t>
+    <t xml:space="preserve">Média prensa automática: minitendência</t>
   </si>
   <si>
     <t xml:space="preserve">Tendência (plot)</t>
   </si>
   <si>
-    <t xml:space="preserve">Carga média: atualizado em</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Carga média: qualidade</t>
+    <t xml:space="preserve">Média prensa automática: atualizado às</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Média prensa automática: qualidade</t>
   </si>
   <si>
     <t xml:space="preserve">`VAL` no arquivo: trocar pelo atributo de qualidade (Parte B)</t>
@@ -130,13 +124,19 @@
     <t xml:space="preserve">Desvio padrão: minitendência</t>
   </si>
   <si>
-    <t xml:space="preserve">Desvio padrão: atualizado em</t>
+    <t xml:space="preserve">Desvio padrão: atualizado às</t>
   </si>
   <si>
     <t xml:space="preserve">Desvio padrão: qualidade</t>
   </si>
   <si>
-    <t xml:space="preserve">Compressão MES: último resultado</t>
+    <t xml:space="preserve">Composto 2 h: prensa automática</t>
+  </si>
+  <si>
+    <t xml:space="preserve">307-GI-001-C2H</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Composto 2 h: laboratório (MES)</t>
   </si>
   <si>
     <t xml:space="preserve">M4710050020-0031-HHLFU</t>
@@ -145,31 +145,58 @@
     <t xml:space="preserve">IP_MESVALOR</t>
   </si>
   <si>
-    <t xml:space="preserve">Compressão MES: horário do resultado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Modo do cortador 07CR001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">U04-07CR001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IP_PIDMAP03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Modo do cortador 07CR002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">U04-07CR002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tendência principal da carga média</t>
-  </si>
-  <si>
-    <t xml:space="preserve">307-GI-001 e M4710050020-0031-HHLFU (ver Parte F)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Faixa menor que 200 (Atenção)</t>
+    <t xml:space="preserve">Composto 2 h: fim da janela</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Composto 2 h: diferença prensa menos laboratório</t>
+  </si>
+  <si>
+    <t xml:space="preserve">307-GI-001-DIF2H</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tendência: composto da prensa x composto do laboratório</t>
+  </si>
+  <si>
+    <t xml:space="preserve">307-GI-001, 307-GI-001-C2H e M4710050020-0031-HHLFU</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cortes do composto: hora do corte 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">307-GI-001-CORTE1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cortes do composto: hora do corte 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">307-GI-001-CORTE2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cortes do composto: hora do corte 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">307-GI-001-CORTE3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cortes do composto: hora do corte 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">307-GI-001-CORTE4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cortes do composto: resultado do corte 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cortes do composto: resultado do corte 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cortes do composto: resultado do corte 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cortes do composto: resultado do corte 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pelotas abaixo de 200 daN</t>
   </si>
   <si>
     <t xml:space="preserve">307-QI-003</t>
@@ -178,13 +205,13 @@
     <t xml:space="preserve">IP_DISCRETEMAP no arquivo: **conferir** (Parte B)</t>
   </si>
   <si>
-    <t xml:space="preserve">Faixa menor que 150 (Alerta)</t>
+    <t xml:space="preserve">Pelotas abaixo de 150 daN</t>
   </si>
   <si>
     <t xml:space="preserve">307-QI-002</t>
   </si>
   <si>
-    <t xml:space="preserve">Faixa menor que 100 (Crítico)</t>
+    <t xml:space="preserve">Pelotas abaixo de 100 daN</t>
   </si>
   <si>
     <t xml:space="preserve">307-QI-001</t>
@@ -612,7 +639,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N23"/>
+  <dimension ref="A1:N30"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -739,28 +766,34 @@
       <c r="C6" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
+      <c r="D6" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>23</v>
+      </c>
       <c r="G6" s="6" t="n">
-        <v>1</v>
+        <v>42.75</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>0.48</v>
+        <v>1.03</v>
       </c>
       <c r="I6" s="6" t="n">
         <v>6.25</v>
       </c>
       <c r="J6" s="6" t="n">
-        <v>1.75</v>
+        <v>0.81</v>
       </c>
       <c r="K6" s="7" t="n">
         <f aca="false">ROUND(G6*$F$2,2)</f>
-        <v>1</v>
+        <v>42.75</v>
       </c>
       <c r="L6" s="7" t="n">
         <f aca="false">ROUND(H6*$F$2,2)</f>
-        <v>0.48</v>
+        <v>1.03</v>
       </c>
       <c r="M6" s="7" t="n">
         <f aca="false">ROUND(I6*$F$2,2)</f>
@@ -768,7 +801,7 @@
       </c>
       <c r="N6" s="7" t="n">
         <f aca="false">ROUND(J6*$F$2,2)</f>
-        <v>1.75</v>
+        <v>0.81</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -776,47 +809,47 @@
         <v>2</v>
       </c>
       <c r="B7" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="E7" s="3" t="s">
         <v>22</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>24</v>
       </c>
       <c r="F7" s="3" t="s">
         <v>25</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>42.75</v>
+        <v>1.78</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>1.31</v>
+        <v>5.47</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>6.25</v>
+        <v>6.41</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>0.81</v>
+        <v>2.63</v>
       </c>
       <c r="K7" s="7" t="n">
         <f aca="false">ROUND(G7*$F$2,2)</f>
-        <v>42.75</v>
+        <v>1.78</v>
       </c>
       <c r="L7" s="7" t="n">
         <f aca="false">ROUND(H7*$F$2,2)</f>
-        <v>1.31</v>
+        <v>5.47</v>
       </c>
       <c r="M7" s="7" t="n">
         <f aca="false">ROUND(I7*$F$2,2)</f>
-        <v>6.25</v>
+        <v>6.41</v>
       </c>
       <c r="N7" s="7" t="n">
         <f aca="false">ROUND(J7*$F$2,2)</f>
-        <v>0.81</v>
+        <v>2.63</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -827,44 +860,40 @@
         <v>26</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>27</v>
-      </c>
+        <v>21</v>
+      </c>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
       <c r="G8" s="6" t="n">
-        <v>1.78</v>
+        <v>11.66</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>5.25</v>
+        <v>5.97</v>
       </c>
       <c r="I8" s="6" t="n">
-        <v>6.41</v>
+        <v>4.38</v>
       </c>
       <c r="J8" s="6" t="n">
-        <v>2.63</v>
+        <v>2.81</v>
       </c>
       <c r="K8" s="7" t="n">
         <f aca="false">ROUND(G8*$F$2,2)</f>
-        <v>1.78</v>
+        <v>11.66</v>
       </c>
       <c r="L8" s="7" t="n">
         <f aca="false">ROUND(H8*$F$2,2)</f>
-        <v>5.25</v>
+        <v>5.97</v>
       </c>
       <c r="M8" s="7" t="n">
         <f aca="false">ROUND(I8*$F$2,2)</f>
-        <v>6.41</v>
+        <v>4.38</v>
       </c>
       <c r="N8" s="7" t="n">
         <f aca="false">ROUND(J8*$F$2,2)</f>
-        <v>2.63</v>
+        <v>2.81</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -875,40 +904,44 @@
         <v>28</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="D9" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F9" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
       <c r="G9" s="6" t="n">
-        <v>11.78</v>
+        <v>4.66</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>5.44</v>
+        <v>9.69</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>4.69</v>
+        <v>5.16</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>3.13</v>
+        <v>0.69</v>
       </c>
       <c r="K9" s="7" t="n">
         <f aca="false">ROUND(G9*$F$2,2)</f>
-        <v>11.78</v>
+        <v>4.66</v>
       </c>
       <c r="L9" s="7" t="n">
         <f aca="false">ROUND(H9*$F$2,2)</f>
-        <v>5.44</v>
+        <v>9.69</v>
       </c>
       <c r="M9" s="7" t="n">
         <f aca="false">ROUND(I9*$F$2,2)</f>
-        <v>4.69</v>
+        <v>5.16</v>
       </c>
       <c r="N9" s="7" t="n">
         <f aca="false">ROUND(J9*$F$2,2)</f>
-        <v>3.13</v>
+        <v>0.69</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -916,43 +949,43 @@
         <v>5</v>
       </c>
       <c r="B10" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F10" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C10" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>25</v>
-      </c>
       <c r="G10" s="6" t="n">
-        <v>4.8</v>
+        <v>12.75</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>9.53</v>
+        <v>9.69</v>
       </c>
       <c r="I10" s="6" t="n">
-        <v>5.16</v>
+        <v>2.5</v>
       </c>
       <c r="J10" s="6" t="n">
         <v>0.69</v>
       </c>
       <c r="K10" s="7" t="n">
         <f aca="false">ROUND(G10*$F$2,2)</f>
-        <v>4.8</v>
+        <v>12.75</v>
       </c>
       <c r="L10" s="7" t="n">
         <f aca="false">ROUND(H10*$F$2,2)</f>
-        <v>9.53</v>
+        <v>9.69</v>
       </c>
       <c r="M10" s="7" t="n">
         <f aca="false">ROUND(I10*$F$2,2)</f>
-        <v>5.16</v>
+        <v>2.5</v>
       </c>
       <c r="N10" s="7" t="n">
         <f aca="false">ROUND(J10*$F$2,2)</f>
@@ -967,44 +1000,44 @@
         <v>31</v>
       </c>
       <c r="C11" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E11" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D11" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>24</v>
-      </c>
       <c r="F11" s="3" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>12.83</v>
+        <v>18.22</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>9.53</v>
+        <v>5.47</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>2.81</v>
+        <v>6.41</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>0.69</v>
+        <v>2.63</v>
       </c>
       <c r="K11" s="7" t="n">
         <f aca="false">ROUND(G11*$F$2,2)</f>
-        <v>12.83</v>
+        <v>18.22</v>
       </c>
       <c r="L11" s="7" t="n">
         <f aca="false">ROUND(H11*$F$2,2)</f>
-        <v>9.53</v>
+        <v>5.47</v>
       </c>
       <c r="M11" s="7" t="n">
         <f aca="false">ROUND(I11*$F$2,2)</f>
-        <v>2.81</v>
+        <v>6.41</v>
       </c>
       <c r="N11" s="7" t="n">
         <f aca="false">ROUND(J11*$F$2,2)</f>
-        <v>0.69</v>
+        <v>2.63</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1015,44 +1048,40 @@
         <v>33</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>27</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
       <c r="G12" s="6" t="n">
-        <v>18.66</v>
+        <v>28.09</v>
       </c>
       <c r="H12" s="6" t="n">
-        <v>5.25</v>
+        <v>5.97</v>
       </c>
       <c r="I12" s="6" t="n">
-        <v>6.41</v>
+        <v>4.38</v>
       </c>
       <c r="J12" s="6" t="n">
-        <v>2.63</v>
+        <v>2.81</v>
       </c>
       <c r="K12" s="7" t="n">
         <f aca="false">ROUND(G12*$F$2,2)</f>
-        <v>18.66</v>
+        <v>28.09</v>
       </c>
       <c r="L12" s="7" t="n">
         <f aca="false">ROUND(H12*$F$2,2)</f>
-        <v>5.25</v>
+        <v>5.97</v>
       </c>
       <c r="M12" s="7" t="n">
         <f aca="false">ROUND(I12*$F$2,2)</f>
-        <v>6.41</v>
+        <v>4.38</v>
       </c>
       <c r="N12" s="7" t="n">
         <f aca="false">ROUND(J12*$F$2,2)</f>
-        <v>2.63</v>
+        <v>2.81</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1060,43 +1089,47 @@
         <v>8</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3"/>
+        <v>32</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>23</v>
+      </c>
       <c r="G13" s="6" t="n">
-        <v>28.66</v>
+        <v>21.1</v>
       </c>
       <c r="H13" s="6" t="n">
-        <v>5.44</v>
+        <v>9.69</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>4.69</v>
+        <v>5.16</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>3.13</v>
+        <v>0.69</v>
       </c>
       <c r="K13" s="7" t="n">
         <f aca="false">ROUND(G13*$F$2,2)</f>
-        <v>28.66</v>
+        <v>21.1</v>
       </c>
       <c r="L13" s="7" t="n">
         <f aca="false">ROUND(H13*$F$2,2)</f>
-        <v>5.44</v>
+        <v>9.69</v>
       </c>
       <c r="M13" s="7" t="n">
         <f aca="false">ROUND(I13*$F$2,2)</f>
-        <v>4.69</v>
+        <v>5.16</v>
       </c>
       <c r="N13" s="7" t="n">
         <f aca="false">ROUND(J13*$F$2,2)</f>
-        <v>3.13</v>
+        <v>0.69</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1104,43 +1137,43 @@
         <v>9</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C14" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E14" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D14" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>24</v>
-      </c>
       <c r="F14" s="3" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>21.68</v>
+        <v>29.18</v>
       </c>
       <c r="H14" s="6" t="n">
-        <v>9.53</v>
+        <v>9.69</v>
       </c>
       <c r="I14" s="6" t="n">
-        <v>5.16</v>
+        <v>2.5</v>
       </c>
       <c r="J14" s="6" t="n">
         <v>0.69</v>
       </c>
       <c r="K14" s="7" t="n">
         <f aca="false">ROUND(G14*$F$2,2)</f>
-        <v>21.68</v>
+        <v>29.18</v>
       </c>
       <c r="L14" s="7" t="n">
         <f aca="false">ROUND(H14*$F$2,2)</f>
-        <v>9.53</v>
+        <v>9.69</v>
       </c>
       <c r="M14" s="7" t="n">
         <f aca="false">ROUND(I14*$F$2,2)</f>
-        <v>5.16</v>
+        <v>2.5</v>
       </c>
       <c r="N14" s="7" t="n">
         <f aca="false">ROUND(J14*$F$2,2)</f>
@@ -1152,47 +1185,47 @@
         <v>10</v>
       </c>
       <c r="B15" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D15" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="E15" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D15" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="E15" s="3" t="s">
-        <v>24</v>
-      </c>
       <c r="F15" s="3" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="G15" s="6" t="n">
-        <v>29.7</v>
+        <v>34.66</v>
       </c>
       <c r="H15" s="6" t="n">
-        <v>9.53</v>
+        <v>5.97</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>2.81</v>
+        <v>5.63</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>0.69</v>
+        <v>2.19</v>
       </c>
       <c r="K15" s="7" t="n">
         <f aca="false">ROUND(G15*$F$2,2)</f>
-        <v>29.7</v>
+        <v>34.66</v>
       </c>
       <c r="L15" s="7" t="n">
         <f aca="false">ROUND(H15*$F$2,2)</f>
-        <v>9.53</v>
+        <v>5.97</v>
       </c>
       <c r="M15" s="7" t="n">
         <f aca="false">ROUND(I15*$F$2,2)</f>
-        <v>2.81</v>
+        <v>5.63</v>
       </c>
       <c r="N15" s="7" t="n">
         <f aca="false">ROUND(J15*$F$2,2)</f>
-        <v>0.69</v>
+        <v>2.19</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1203,7 +1236,7 @@
         <v>38</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D16" s="3" t="s">
         <v>39</v>
@@ -1212,35 +1245,35 @@
         <v>40</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="G16" s="6" t="n">
-        <v>35.53</v>
+        <v>43.71</v>
       </c>
       <c r="H16" s="6" t="n">
-        <v>5.81</v>
+        <v>5.97</v>
       </c>
       <c r="I16" s="6" t="n">
-        <v>5.31</v>
+        <v>4.06</v>
       </c>
       <c r="J16" s="6" t="n">
-        <v>2.63</v>
+        <v>2.19</v>
       </c>
       <c r="K16" s="7" t="n">
         <f aca="false">ROUND(G16*$F$2,2)</f>
-        <v>35.53</v>
+        <v>43.71</v>
       </c>
       <c r="L16" s="7" t="n">
         <f aca="false">ROUND(H16*$F$2,2)</f>
-        <v>5.81</v>
+        <v>5.97</v>
       </c>
       <c r="M16" s="7" t="n">
         <f aca="false">ROUND(I16*$F$2,2)</f>
-        <v>5.31</v>
+        <v>4.06</v>
       </c>
       <c r="N16" s="7" t="n">
         <f aca="false">ROUND(J16*$F$2,2)</f>
-        <v>2.63</v>
+        <v>2.19</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1251,40 +1284,40 @@
         <v>41</v>
       </c>
       <c r="C17" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="E17" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D17" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>40</v>
-      </c>
       <c r="F17" s="3" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="G17" s="6" t="n">
-        <v>43.53</v>
+        <v>37.53</v>
       </c>
       <c r="H17" s="6" t="n">
-        <v>8.69</v>
+        <v>9.06</v>
       </c>
       <c r="I17" s="6" t="n">
-        <v>4.69</v>
+        <v>3.94</v>
       </c>
       <c r="J17" s="6" t="n">
         <v>0.69</v>
       </c>
       <c r="K17" s="7" t="n">
         <f aca="false">ROUND(G17*$F$2,2)</f>
-        <v>43.53</v>
+        <v>37.53</v>
       </c>
       <c r="L17" s="7" t="n">
         <f aca="false">ROUND(H17*$F$2,2)</f>
-        <v>8.69</v>
+        <v>9.06</v>
       </c>
       <c r="M17" s="7" t="n">
         <f aca="false">ROUND(I17*$F$2,2)</f>
-        <v>4.69</v>
+        <v>3.94</v>
       </c>
       <c r="N17" s="7" t="n">
         <f aca="false">ROUND(J17*$F$2,2)</f>
@@ -1299,44 +1332,44 @@
         <v>42</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D18" s="3" t="s">
         <v>43</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>44</v>
+        <v>22</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>44.78</v>
+        <v>44.03</v>
       </c>
       <c r="H18" s="6" t="n">
-        <v>11.22</v>
+        <v>9.06</v>
       </c>
       <c r="I18" s="6" t="n">
-        <v>3.44</v>
+        <v>1.75</v>
       </c>
       <c r="J18" s="6" t="n">
-        <v>0.81</v>
+        <v>0.69</v>
       </c>
       <c r="K18" s="7" t="n">
         <f aca="false">ROUND(G18*$F$2,2)</f>
-        <v>44.78</v>
+        <v>44.03</v>
       </c>
       <c r="L18" s="7" t="n">
         <f aca="false">ROUND(H18*$F$2,2)</f>
-        <v>11.22</v>
+        <v>9.06</v>
       </c>
       <c r="M18" s="7" t="n">
         <f aca="false">ROUND(I18*$F$2,2)</f>
-        <v>3.44</v>
+        <v>1.75</v>
       </c>
       <c r="N18" s="7" t="n">
         <f aca="false">ROUND(J18*$F$2,2)</f>
-        <v>0.81</v>
+        <v>0.69</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1344,47 +1377,43 @@
         <v>14</v>
       </c>
       <c r="B19" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D19" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="C19" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D19" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="F19" s="3" t="s">
-        <v>27</v>
-      </c>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
       <c r="G19" s="6" t="n">
-        <v>44.78</v>
+        <v>3.16</v>
       </c>
       <c r="H19" s="6" t="n">
-        <v>12.47</v>
+        <v>15.06</v>
       </c>
       <c r="I19" s="6" t="n">
-        <v>3.44</v>
+        <v>30.94</v>
       </c>
       <c r="J19" s="6" t="n">
-        <v>0.81</v>
+        <v>17.5</v>
       </c>
       <c r="K19" s="7" t="n">
         <f aca="false">ROUND(G19*$F$2,2)</f>
-        <v>44.78</v>
+        <v>3.16</v>
       </c>
       <c r="L19" s="7" t="n">
         <f aca="false">ROUND(H19*$F$2,2)</f>
-        <v>12.47</v>
+        <v>15.06</v>
       </c>
       <c r="M19" s="7" t="n">
         <f aca="false">ROUND(I19*$F$2,2)</f>
-        <v>3.44</v>
+        <v>30.94</v>
       </c>
       <c r="N19" s="7" t="n">
         <f aca="false">ROUND(J19*$F$2,2)</f>
-        <v>0.81</v>
+        <v>17.5</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1392,43 +1421,47 @@
         <v>15</v>
       </c>
       <c r="B20" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D20" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C20" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="D20" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="E20" s="3"/>
-      <c r="F20" s="3"/>
+      <c r="E20" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>23</v>
+      </c>
       <c r="G20" s="6" t="n">
-        <v>3.03</v>
+        <v>37.72</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>14.63</v>
+        <v>15.8</v>
       </c>
       <c r="I20" s="6" t="n">
-        <v>29.63</v>
+        <v>2.5</v>
       </c>
       <c r="J20" s="6" t="n">
-        <v>18</v>
+        <v>0.75</v>
       </c>
       <c r="K20" s="7" t="n">
         <f aca="false">ROUND(G20*$F$2,2)</f>
-        <v>3.03</v>
+        <v>37.72</v>
       </c>
       <c r="L20" s="7" t="n">
         <f aca="false">ROUND(H20*$F$2,2)</f>
-        <v>14.63</v>
+        <v>15.8</v>
       </c>
       <c r="M20" s="7" t="n">
         <f aca="false">ROUND(I20*$F$2,2)</f>
-        <v>29.63</v>
+        <v>2.5</v>
       </c>
       <c r="N20" s="7" t="n">
         <f aca="false">ROUND(J20*$F$2,2)</f>
-        <v>18</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1436,47 +1469,47 @@
         <v>16</v>
       </c>
       <c r="B21" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D21" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="C21" s="3" t="s">
+      <c r="E21" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D21" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="E21" s="3" t="s">
-        <v>51</v>
-      </c>
       <c r="F21" s="3" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="G21" s="6" t="n">
-        <v>44.31</v>
+        <v>37.72</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>19.91</v>
+        <v>17.05</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>3.25</v>
+        <v>2.5</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="K21" s="7" t="n">
         <f aca="false">ROUND(G21*$F$2,2)</f>
-        <v>44.31</v>
+        <v>37.72</v>
       </c>
       <c r="L21" s="7" t="n">
         <f aca="false">ROUND(H21*$F$2,2)</f>
-        <v>19.91</v>
+        <v>17.05</v>
       </c>
       <c r="M21" s="7" t="n">
         <f aca="false">ROUND(I21*$F$2,2)</f>
-        <v>3.25</v>
+        <v>2.5</v>
       </c>
       <c r="N21" s="7" t="n">
         <f aca="false">ROUND(J21*$F$2,2)</f>
-        <v>1</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1484,47 +1517,47 @@
         <v>17</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C22" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="E22" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D22" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="E22" s="3" t="s">
-        <v>51</v>
-      </c>
       <c r="F22" s="3" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="G22" s="6" t="n">
-        <v>44.31</v>
+        <v>37.72</v>
       </c>
       <c r="H22" s="6" t="n">
-        <v>24.53</v>
+        <v>18.3</v>
       </c>
       <c r="I22" s="6" t="n">
-        <v>3.25</v>
+        <v>2.5</v>
       </c>
       <c r="J22" s="6" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="K22" s="7" t="n">
         <f aca="false">ROUND(G22*$F$2,2)</f>
-        <v>44.31</v>
+        <v>37.72</v>
       </c>
       <c r="L22" s="7" t="n">
         <f aca="false">ROUND(H22*$F$2,2)</f>
-        <v>24.53</v>
+        <v>18.3</v>
       </c>
       <c r="M22" s="7" t="n">
         <f aca="false">ROUND(I22*$F$2,2)</f>
-        <v>3.25</v>
+        <v>2.5</v>
       </c>
       <c r="N22" s="7" t="n">
         <f aca="false">ROUND(J22*$F$2,2)</f>
-        <v>1</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1532,47 +1565,383 @@
         <v>18</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C23" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="E23" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D23" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="E23" s="3" t="s">
-        <v>51</v>
-      </c>
       <c r="F23" s="3" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="G23" s="6" t="n">
-        <v>44.31</v>
+        <v>37.72</v>
       </c>
       <c r="H23" s="6" t="n">
-        <v>29.16</v>
+        <v>19.55</v>
       </c>
       <c r="I23" s="6" t="n">
-        <v>3.25</v>
+        <v>2.5</v>
       </c>
       <c r="J23" s="6" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="K23" s="7" t="n">
         <f aca="false">ROUND(G23*$F$2,2)</f>
-        <v>44.31</v>
+        <v>37.72</v>
       </c>
       <c r="L23" s="7" t="n">
         <f aca="false">ROUND(H23*$F$2,2)</f>
-        <v>29.16</v>
+        <v>19.55</v>
       </c>
       <c r="M23" s="7" t="n">
         <f aca="false">ROUND(I23*$F$2,2)</f>
-        <v>3.25</v>
+        <v>2.5</v>
       </c>
       <c r="N23" s="7" t="n">
         <f aca="false">ROUND(J23*$F$2,2)</f>
-        <v>1</v>
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F24" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="G24" s="6" t="n">
+        <v>42.09</v>
+      </c>
+      <c r="H24" s="6" t="n">
+        <v>15.77</v>
+      </c>
+      <c r="I24" s="6" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="J24" s="6" t="n">
+        <v>0.81</v>
+      </c>
+      <c r="K24" s="7" t="n">
+        <f aca="false">ROUND(G24*$F$2,2)</f>
+        <v>42.09</v>
+      </c>
+      <c r="L24" s="7" t="n">
+        <f aca="false">ROUND(H24*$F$2,2)</f>
+        <v>15.77</v>
+      </c>
+      <c r="M24" s="7" t="n">
+        <f aca="false">ROUND(I24*$F$2,2)</f>
+        <v>3.75</v>
+      </c>
+      <c r="N24" s="7" t="n">
+        <f aca="false">ROUND(J24*$F$2,2)</f>
+        <v>0.81</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F25" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="G25" s="6" t="n">
+        <v>42.09</v>
+      </c>
+      <c r="H25" s="6" t="n">
+        <v>17.02</v>
+      </c>
+      <c r="I25" s="6" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="J25" s="6" t="n">
+        <v>0.81</v>
+      </c>
+      <c r="K25" s="7" t="n">
+        <f aca="false">ROUND(G25*$F$2,2)</f>
+        <v>42.09</v>
+      </c>
+      <c r="L25" s="7" t="n">
+        <f aca="false">ROUND(H25*$F$2,2)</f>
+        <v>17.02</v>
+      </c>
+      <c r="M25" s="7" t="n">
+        <f aca="false">ROUND(I25*$F$2,2)</f>
+        <v>3.75</v>
+      </c>
+      <c r="N25" s="7" t="n">
+        <f aca="false">ROUND(J25*$F$2,2)</f>
+        <v>0.81</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F26" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="G26" s="6" t="n">
+        <v>42.09</v>
+      </c>
+      <c r="H26" s="6" t="n">
+        <v>18.27</v>
+      </c>
+      <c r="I26" s="6" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="J26" s="6" t="n">
+        <v>0.81</v>
+      </c>
+      <c r="K26" s="7" t="n">
+        <f aca="false">ROUND(G26*$F$2,2)</f>
+        <v>42.09</v>
+      </c>
+      <c r="L26" s="7" t="n">
+        <f aca="false">ROUND(H26*$F$2,2)</f>
+        <v>18.27</v>
+      </c>
+      <c r="M26" s="7" t="n">
+        <f aca="false">ROUND(I26*$F$2,2)</f>
+        <v>3.75</v>
+      </c>
+      <c r="N26" s="7" t="n">
+        <f aca="false">ROUND(J26*$F$2,2)</f>
+        <v>0.81</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F27" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="G27" s="6" t="n">
+        <v>42.09</v>
+      </c>
+      <c r="H27" s="6" t="n">
+        <v>19.52</v>
+      </c>
+      <c r="I27" s="6" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="J27" s="6" t="n">
+        <v>0.81</v>
+      </c>
+      <c r="K27" s="7" t="n">
+        <f aca="false">ROUND(G27*$F$2,2)</f>
+        <v>42.09</v>
+      </c>
+      <c r="L27" s="7" t="n">
+        <f aca="false">ROUND(H27*$F$2,2)</f>
+        <v>19.52</v>
+      </c>
+      <c r="M27" s="7" t="n">
+        <f aca="false">ROUND(I27*$F$2,2)</f>
+        <v>3.75</v>
+      </c>
+      <c r="N27" s="7" t="n">
+        <f aca="false">ROUND(J27*$F$2,2)</f>
+        <v>0.81</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F28" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="G28" s="6" t="n">
+        <v>44.34</v>
+      </c>
+      <c r="H28" s="6" t="n">
+        <v>24.52</v>
+      </c>
+      <c r="I28" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="J28" s="6" t="n">
+        <v>0.94</v>
+      </c>
+      <c r="K28" s="7" t="n">
+        <f aca="false">ROUND(G28*$F$2,2)</f>
+        <v>44.34</v>
+      </c>
+      <c r="L28" s="7" t="n">
+        <f aca="false">ROUND(H28*$F$2,2)</f>
+        <v>24.52</v>
+      </c>
+      <c r="M28" s="7" t="n">
+        <f aca="false">ROUND(I28*$F$2,2)</f>
+        <v>2</v>
+      </c>
+      <c r="N28" s="7" t="n">
+        <f aca="false">ROUND(J28*$F$2,2)</f>
+        <v>0.94</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F29" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="G29" s="6" t="n">
+        <v>44.34</v>
+      </c>
+      <c r="H29" s="6" t="n">
+        <v>25.89</v>
+      </c>
+      <c r="I29" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="J29" s="6" t="n">
+        <v>0.94</v>
+      </c>
+      <c r="K29" s="7" t="n">
+        <f aca="false">ROUND(G29*$F$2,2)</f>
+        <v>44.34</v>
+      </c>
+      <c r="L29" s="7" t="n">
+        <f aca="false">ROUND(H29*$F$2,2)</f>
+        <v>25.89</v>
+      </c>
+      <c r="M29" s="7" t="n">
+        <f aca="false">ROUND(I29*$F$2,2)</f>
+        <v>2</v>
+      </c>
+      <c r="N29" s="7" t="n">
+        <f aca="false">ROUND(J29*$F$2,2)</f>
+        <v>0.94</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="E30" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F30" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="G30" s="6" t="n">
+        <v>44.34</v>
+      </c>
+      <c r="H30" s="6" t="n">
+        <v>27.27</v>
+      </c>
+      <c r="I30" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="J30" s="6" t="n">
+        <v>0.94</v>
+      </c>
+      <c r="K30" s="7" t="n">
+        <f aca="false">ROUND(G30*$F$2,2)</f>
+        <v>44.34</v>
+      </c>
+      <c r="L30" s="7" t="n">
+        <f aca="false">ROUND(H30*$F$2,2)</f>
+        <v>27.27</v>
+      </c>
+      <c r="M30" s="7" t="n">
+        <f aca="false">ROUND(I30*$F$2,2)</f>
+        <v>2</v>
+      </c>
+      <c r="N30" s="7" t="n">
+        <f aca="false">ROUND(J30*$F$2,2)</f>
+        <v>0.94</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Tela v7: kgf/pelota, faixas de compressão e composto com cortes parciais
Unidade em kgf/pelota, quadro renomeado para faixas de compressão,
quantidade de cortes com resultado na janela, regra de média com 1 a 4
cortes na especificação das tags calculadas e contorno do logotipo sem
pontos repetidos.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012cAZJr8EKNEq3XLjv1AThq
</commit_message>
<xml_diff>
--- a/entregaveis/03_aspen/posicoes_objetos.xlsx
+++ b/entregaveis/03_aspen/posicoes_objetos.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="67">
   <si>
     <t xml:space="preserve">Largura da tela no editor, em unidades. O padrão do Aspen é 50; só altere se a tela tiver outro tamanho.</t>
   </si>
@@ -196,7 +196,7 @@
     <t xml:space="preserve">Cortes do composto: resultado do corte 4</t>
   </si>
   <si>
-    <t xml:space="preserve">Pelotas abaixo de 200 daN</t>
+    <t xml:space="preserve">Faixa abaixo de 200 kgf/pelota</t>
   </si>
   <si>
     <t xml:space="preserve">307-QI-003</t>
@@ -205,16 +205,22 @@
     <t xml:space="preserve">IP_DISCRETEMAP no arquivo: **conferir** (Parte B)</t>
   </si>
   <si>
-    <t xml:space="preserve">Pelotas abaixo de 150 daN</t>
+    <t xml:space="preserve">Faixa abaixo de 150 kgf/pelota</t>
   </si>
   <si>
     <t xml:space="preserve">307-QI-002</t>
   </si>
   <si>
-    <t xml:space="preserve">Pelotas abaixo de 100 daN</t>
+    <t xml:space="preserve">Faixa abaixo de 100 kgf/pelota</t>
   </si>
   <si>
     <t xml:space="preserve">307-QI-001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Composto 2 h: cortes com resultado na janela</t>
+  </si>
+  <si>
+    <t xml:space="preserve">307-GI-001-N2H</t>
   </si>
 </sst>
 </file>
@@ -639,7 +645,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N30"/>
+  <dimension ref="A1:N31"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -1820,7 +1826,7 @@
         <v>25</v>
       </c>
       <c r="G28" s="6" t="n">
-        <v>44.34</v>
+        <v>46.03</v>
       </c>
       <c r="H28" s="6" t="n">
         <v>24.52</v>
@@ -1833,7 +1839,7 @@
       </c>
       <c r="K28" s="7" t="n">
         <f aca="false">ROUND(G28*$F$2,2)</f>
-        <v>44.34</v>
+        <v>46.03</v>
       </c>
       <c r="L28" s="7" t="n">
         <f aca="false">ROUND(H28*$F$2,2)</f>
@@ -1868,7 +1874,7 @@
         <v>25</v>
       </c>
       <c r="G29" s="6" t="n">
-        <v>44.34</v>
+        <v>46.03</v>
       </c>
       <c r="H29" s="6" t="n">
         <v>25.89</v>
@@ -1881,7 +1887,7 @@
       </c>
       <c r="K29" s="7" t="n">
         <f aca="false">ROUND(G29*$F$2,2)</f>
-        <v>44.34</v>
+        <v>46.03</v>
       </c>
       <c r="L29" s="7" t="n">
         <f aca="false">ROUND(H29*$F$2,2)</f>
@@ -1916,7 +1922,7 @@
         <v>25</v>
       </c>
       <c r="G30" s="6" t="n">
-        <v>44.34</v>
+        <v>46.03</v>
       </c>
       <c r="H30" s="6" t="n">
         <v>27.27</v>
@@ -1929,7 +1935,7 @@
       </c>
       <c r="K30" s="7" t="n">
         <f aca="false">ROUND(G30*$F$2,2)</f>
-        <v>44.34</v>
+        <v>46.03</v>
       </c>
       <c r="L30" s="7" t="n">
         <f aca="false">ROUND(H30*$F$2,2)</f>
@@ -1942,6 +1948,54 @@
       <c r="N30" s="7" t="n">
         <f aca="false">ROUND(J30*$F$2,2)</f>
         <v>0.94</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="E31" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F31" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="G31" s="6" t="n">
+        <v>40.1</v>
+      </c>
+      <c r="H31" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="I31" s="6" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J31" s="6" t="n">
+        <v>0.69</v>
+      </c>
+      <c r="K31" s="7" t="n">
+        <f aca="false">ROUND(G31*$F$2,2)</f>
+        <v>40.1</v>
+      </c>
+      <c r="L31" s="7" t="n">
+        <f aca="false">ROUND(H31*$F$2,2)</f>
+        <v>10</v>
+      </c>
+      <c r="M31" s="7" t="n">
+        <f aca="false">ROUND(I31*$F$2,2)</f>
+        <v>0.75</v>
+      </c>
+      <c r="N31" s="7" t="n">
+        <f aca="false">ROUND(J31*$F$2,2)</f>
+        <v>0.69</v>
       </c>
     </row>
   </sheetData>

</xml_diff>